<commit_message>
Group B: FS6809 SPEC (FS swivel x FS adjustable stud) + NWO_FS[6] measured on BRENNAN_FS6809-06-06-NWO-FG; OCP closed loop 0 off
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/orfs_tables/DesignTable_FS6809.xlsx
+++ b/tools/_out/groupB_20261021/stage/orfs_tables/DesignTable_FS6809.xlsx
@@ -539,6 +539,9 @@
       <c r="B3" t="n">
         <v>1.29</v>
       </c>
+      <c r="C3" t="n">
+        <v>0.857</v>
+      </c>
       <c r="D3" t="n">
         <v>1.04</v>
       </c>
@@ -585,17 +588,17 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "AAA LGTH" = "1.04" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "N LGTH" = "1.29" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "C1 HEX" = "0.687" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-4 S 0.69 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "C2 HEX" = "0.625" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "JJ FLATS" = "0.562" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "A HOLE" = "0.165" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "B HOLE" = "0.172" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -04 = 0.5625 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "A THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -04 = 0.4375 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "B THREAD" "7/16-20" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "A THREAD" "9/16-18" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "B THREAD" "7/16-20" in the table's format</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: L11@DRIVE] [BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "AAA LGTH" = "1.04" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "N LGTH" = "1.29" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "C1 HEX" = "0.687" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-4 S 0.69 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "C2 HEX" = "0.625" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "JJ FLATS" = "0.562" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "A HOLE" = "0.165" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "B HOLE" = "0.172" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 151.5, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -04 = 0.5625 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "A THREAD" "9/16-18" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -04 = 0.4375 (PLAN.md s2 FS_THR / the -04 thread of every staged ORFS row); = Brennan "B THREAD" "7/16-20" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "A THREAD" "9/16-18" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-04-04-NWO-FG col "B THREAD" "7/16-20" in the table's format</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on AAA LGTH=1.04 vs Air-Way L21=1.29 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5697 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-04-04-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on AAA LGTH=1.04 vs Air-Way L21=1.29 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5697 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-04-04-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6809-04-04-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: L11@DRIVE=N-DT; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -715,6 +718,9 @@
       <c r="B5" t="n">
         <v>1.6</v>
       </c>
+      <c r="C5" t="n">
+        <v>1.06</v>
+      </c>
       <c r="D5" t="n">
         <v>1.49</v>
       </c>
@@ -761,17 +767,17 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "AAA LGTH" = "1.49" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "N LGTH" = "1.60" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "C1 HEX" = "0.938" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-8 S 0.94 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "C2 HEX" = "0.938" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "JJ FLATS" = "0.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "A HOLE" = "0.358" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "B HOLE" = "0.378" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -08 = 0.8125 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "A THREAD" "13/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -08 = 0.75 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "B THREAD" "3/4-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "A THREAD" "13/16-16" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "B THREAD" "3/4-16" in the table's format</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: L11@DRIVE] [BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "AAA LGTH" = "1.49" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "N LGTH" = "1.60" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "C1 HEX" = "0.938" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-8 S 0.94 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "C2 HEX" = "0.938" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "JJ FLATS" = "0.750" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "A HOLE" = "0.358" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "B HOLE" = "0.378" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 171.6, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -08 = 0.8125 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "A THREAD" "13/16-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -08 = 0.75 (PLAN.md s2 FS_THR / the -08 thread of every staged ORFS row); = Brennan "B THREAD" "3/4-16" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "A THREAD" "13/16-16" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-08-08-NWO-FG col "B THREAD" "3/4-16" in the table's format</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on JJ FLATS=0.750 vs Air-Way S2=0.56 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5699 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-08-08-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on JJ FLATS=0.750 vs Air-Way S2=0.56 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5699 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-08-08-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6809-08-08-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: L11@DRIVE=N-DT; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -804,6 +810,9 @@
       <c r="B6" t="n">
         <v>1.97</v>
       </c>
+      <c r="C6" t="n">
+        <v>1.336</v>
+      </c>
       <c r="D6" t="n">
         <v>1.62</v>
       </c>
@@ -850,17 +859,17 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "AAA LGTH" = "1.62" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "N LGTH" = "1.97" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "C1 HEX" = "1.125" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-10 S 1.13 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "C2 HEX" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "JJ FLATS" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "A HOLE" = "0.453" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "B HOLE" = "0.484" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -10 = 1.0 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "A THREAD" "1-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -10 = 0.875 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "B THREAD" "7/8-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "A THREAD" "1-14" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "B THREAD" "7/8-14" in the table's format</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: L11@DRIVE] [BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "AAA LGTH" = "1.62" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "N LGTH" = "1.97" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "C1 HEX" = "1.125" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-10 S 1.13 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "C2 HEX" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "JJ FLATS" = "1.062" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "A HOLE" = "0.453" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "B HOLE" = "0.484" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 181.7, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -10 = 1.0 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "A THREAD" "1-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -10 = 0.875 (PLAN.md s2 FS_THR / the -10 thread of every staged ORFS row); = Brennan "B THREAD" "7/8-14" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "A THREAD" "1-14" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-10-10-NWO-FG col "B THREAD" "7/8-14" in the table's format</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on JJ FLATS=1.062 vs Air-Way S2=0.94 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5700 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-10-10-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>forged (-FG): Air-Way non-forged row differs from Brennan forged on JJ FLATS=1.062 vs Air-Way S2=0.94 - stays MISSING (user 2026-10-15) | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5700 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-10-10-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6809-10-10-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: L11@DRIVE=N-DT; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -893,6 +902,9 @@
       <c r="B7" t="n">
         <v>2.17</v>
       </c>
+      <c r="C7" t="n">
+        <v>1.443</v>
+      </c>
       <c r="D7" t="n">
         <v>1.82</v>
       </c>
@@ -939,17 +951,17 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>ASSUMED</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>[BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "AAA LGTH" = "1.82" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "N LGTH" = "2.17" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "C1 HEX" = "1.375" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-12 S 1.38 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "C2 HEX" = "1.375" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "JJ FLATS" = "1.188" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "A HOLE" = "0.547" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "B HOLE" = "0.609" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -12 = 1.1875 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "A THREAD" "1-3/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -12 = 1.0625 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "B THREAD" "1-1/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "A THREAD" "1-3/16-12" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "B THREAD" "1-1/16-12" in the table's format</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: L11@DRIVE] [BRENNAN-ONLY 2026-10-18] not built: forged part where Air-Way and Brennan do not match on every cell (user 2026-10-15: the rest stay MISSING) -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"): L21@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "AAA LGTH" = "1.82" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel leg crossing -&gt; nut face; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; L10@DRIVE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "N LGTH" = "2.17" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - adjustable stud tip -&gt; crossing; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; SHEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "C1 HEX" = "1.375" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; Q-FS-NUT: = Air-Way FF318-12 S 1.38 to rounding; S3HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "C2 HEX" = "1.375" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - lock nut hex; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; S2HEX@HEX: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "JJ FLATS" = "1.188" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - forged flats; mapping: same-table check: 3/3 rows with an Air-Way value agree to rounding; D19@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "A HOLE" = "0.547" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - swivel-end bore; mapping: same-table check: 2/3 rows with an Air-Way value agree to rounding (1 differ, e.g. FS6809-16-16-NWO-FG 0.79 vs 0.783); D20@BORE: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "B HOLE" = "0.609" (07_RAW_EXTRACTS/brennan_catalogs/ORFS Catalog.pdf; tools/_out/brennan_catalog_20261001/catalog_verified.json, line_y 191.8, page verified True) [Brennan = yes 2026-10-18] - stud-end bore; mapping: same-table check: 1/3 rows with an Air-Way value agree to rounding (2 differ, e.g. FS6809-16-16-NWO-FG 0.85 vs 0.811); THDMAJ_D@DRIVE: end library: face-seal (SAE J1453) thread FS_THR of dash -12 = 1.1875 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "A THREAD" "1-3/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; THDMAJ_N@DRIVE: end library: straight (UN/UNF) thread of dash -12 = 1.0625 (PLAN.md s2 FS_THR / the -12 thread of every staged ORFS row); = Brennan "B THREAD" "1-1/16-12" of this row [Q-TRANSFER-ENDLIB yes 2026-10-08]; $PRP@Thread_D: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "A THREAD" "1-3/16-12" in the table's format; $PRP@Thread_N: Brennan ORFS catalog p11 table ORFS-p011-t01 "FS6809-NWO-FG FFSS-MAORB 90 DEG ELBOW" row FS6809-12-12-NWO-FG col "B THREAD" "1-1/16-12" in the table's format</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>forged (-FG): Brennan p11 prints it but Air-Way has no non-forged row - Brennan-only stays MISSING | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5701 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-12-12-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library)</t>
+          <t>forged (-FG): Brennan p11 prints it but Air-Way has no non-forged row - Brennan-only stays MISSING | forged (-FG): the Air-Way NON-forged series FF6809 is used only where Brennan FS6809-NWO-FG prints the same value in every compared cell (user 2026-10-15); forged body shape from Brennan (shape only) | OMi parts file row 5701 (no dimensions) | 2026-10-18 Brennan = yes (wave 3 ORFS, staged, not shipped): sizes from Brennan ORFS p11 FS6809-12-12-NWO-FG ($PRP@DimSource BRENNAN; to undo clear the BRENNAN cells and regenerate); threads by dash (end library) | Brennan CAD record FS6809-12-12-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: L11@DRIVE=N-DT; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">

</xml_diff>